<commit_message>
Update Kho gửi phòng SX-BH 03_2026.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/Thiết bị kho gửi/2026/Kho gửi phòng SX-BH 03_2026.xlsx
+++ b/5. Other/Thiết bị kho gửi/2026/Kho gửi phòng SX-BH 03_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\Thiết bị kho gửi\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A664EB-5D16-4792-802C-1C460ABE2F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FBCED9-1138-4597-BA27-FCCD753158AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nhập xuất tồn" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="79">
   <si>
     <t>VNSH01</t>
   </si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>dlrantai</t>
+  </si>
+  <si>
+    <t>Đã trả (02/03/26)</t>
   </si>
 </sst>
 </file>
@@ -537,10 +540,10 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1075,18 +1078,18 @@
       </c>
       <c r="E4" s="3">
         <f>Xuất!AH5+Huỷ!AH4</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" s="3">
         <f>C4+D4-E4</f>
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="G4" s="4">
         <v>16</v>
       </c>
       <c r="H4" s="3">
         <f t="shared" ref="H4:H22" si="0">F4-G4</f>
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1683,11 +1686,11 @@
       </c>
       <c r="E24" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24" s="3">
         <f>SUM(F3:F23)</f>
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G24" s="3">
         <f t="shared" si="2"/>
@@ -1695,7 +1698,7 @@
       </c>
       <c r="H24" s="3">
         <f>SUM(H3:H23)</f>
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -3021,7 +3024,9 @@
         <v>1</v>
       </c>
       <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="D5" s="5">
+        <v>3</v>
+      </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
@@ -3053,7 +3058,7 @@
       <c r="AG5" s="5"/>
       <c r="AH5" s="5">
         <f t="shared" ref="AH5:AH18" si="0">SUM(C5:AG5)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -5235,7 +5240,7 @@
       <c r="G21" s="16"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
+      <c r="A22" s="33"/>
       <c r="B22" s="15" t="s">
         <v>65</v>
       </c>
@@ -5250,7 +5255,7 @@
       <c r="G22" s="16"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="33"/>
+      <c r="A23" s="34"/>
       <c r="B23" s="15" t="s">
         <v>67</v>
       </c>
@@ -5282,7 +5287,7 @@
       <c r="G24" s="16"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
+      <c r="A25" s="33"/>
       <c r="B25" s="15" t="s">
         <v>64</v>
       </c>
@@ -5297,7 +5302,7 @@
       <c r="G25" s="16"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="33"/>
+      <c r="A26" s="34"/>
       <c r="B26" s="15" t="s">
         <v>14</v>
       </c>
@@ -5333,7 +5338,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="33"/>
+      <c r="A28" s="34"/>
       <c r="B28" s="15" t="s">
         <v>50</v>
       </c>
@@ -5367,7 +5372,7 @@
       <c r="G29" s="16"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="34"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="15" t="s">
         <v>71</v>
       </c>
@@ -5382,7 +5387,7 @@
       <c r="G30" s="16"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="33"/>
+      <c r="A31" s="34"/>
       <c r="B31" s="15" t="s">
         <v>50</v>
       </c>
@@ -5433,7 +5438,7 @@
       <c r="G33" s="16"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
+      <c r="A34" s="33"/>
       <c r="B34" s="15" t="s">
         <v>50</v>
       </c>
@@ -5448,7 +5453,7 @@
       <c r="G34" s="16"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
+      <c r="A35" s="33"/>
       <c r="B35" s="15" t="s">
         <v>14</v>
       </c>
@@ -5458,12 +5463,12 @@
         <v>2</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="G35" s="16"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
+      <c r="A36" s="33"/>
       <c r="B36" s="15" t="s">
         <v>76</v>
       </c>
@@ -5488,17 +5493,23 @@
         <v>1</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="G37" s="16"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="14"/>
-      <c r="B38" s="15"/>
+      <c r="A38" s="34"/>
+      <c r="B38" s="15" t="s">
+        <v>62</v>
+      </c>
       <c r="C38" s="15"/>
       <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
+      <c r="E38" s="15">
+        <v>50</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>69</v>
+      </c>
       <c r="G38" s="16"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -5613,7 +5624,6 @@
   </sheetData>
   <autoFilter ref="A1:F7" xr:uid="{171653DB-B967-4059-9CE3-FD13B7B63DBC}"/>
   <mergeCells count="12">
-    <mergeCell ref="A33:A37"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A7"/>
@@ -5625,6 +5635,7 @@
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A33:A38"/>
   </mergeCells>
   <conditionalFormatting sqref="D2:F1000">
     <cfRule type="expression" dxfId="1" priority="1">
@@ -5735,18 +5746,18 @@
       </c>
       <c r="E4" s="3">
         <f>SUM('Nhập xuất tồn'!E4)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" s="3">
         <f>SUM(C4+D4-E4)</f>
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="G4" s="4">
         <v>14</v>
       </c>
       <c r="H4" s="3">
         <f>SUM(F4-G4)</f>
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6189,11 +6200,11 @@
       </c>
       <c r="E19" s="10">
         <f>SUM(E3:E17)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" s="10">
         <f>SUM(F3:F18)</f>
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G19" s="11">
         <f>SUM(G3:G17)</f>
@@ -6201,7 +6212,7 @@
       </c>
       <c r="H19" s="10">
         <f>SUM(H3:H18)</f>
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>